<commit_message>
feat: actualizar plantilla de preliquidacion en analytica
</commit_message>
<xml_diff>
--- a/liquidacion/analytica/Report/PreLiquidacion.xlsx
+++ b/liquidacion/analytica/Report/PreLiquidacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ProBook\source\acopio\acopio-liquidacion-api\Acopio.Liquidaciones.Apis\Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\minersoft\acopio-project-configuration\liquidacion\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DC9B68-DA1E-44E3-883A-5790DD0F99C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD5A92D-8B09-436A-8515-6929C4720338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,80 +20,104 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>Miner Soft S. A. C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROPUESTA DE VALORIZACION DE MINERAL </t>
-  </si>
-  <si>
-    <t>Mineral</t>
-  </si>
-  <si>
-    <t>TMH</t>
-  </si>
-  <si>
-    <t>TMS</t>
-  </si>
-  <si>
-    <t>%H2O</t>
-  </si>
-  <si>
-    <t>Maquila</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ley Oz/Tc </t>
-  </si>
-  <si>
-    <t>% Recup.</t>
-  </si>
-  <si>
-    <t>Fecha Ingreso</t>
-  </si>
-  <si>
-    <t>GRR</t>
-  </si>
-  <si>
-    <t>GRT</t>
-  </si>
-  <si>
-    <t>Unidad Medida</t>
-  </si>
-  <si>
-    <t>Tipo mineral</t>
-  </si>
-  <si>
-    <t>Procedencia</t>
-  </si>
-  <si>
-    <t>Inter US$</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Lote</t>
-  </si>
-  <si>
-    <t>Proveedor</t>
-  </si>
-  <si>
-    <t>Ruc</t>
-  </si>
-  <si>
-    <t>Consumos</t>
-  </si>
-  <si>
-    <t>Precio</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+  <si>
+    <t>LIQUIDACION DE VENTA DE ACOPIO [el año  registro de la liquidación masiva]</t>
+  </si>
+  <si>
+    <t>Analytica Mineral Services Sac</t>
+  </si>
+  <si>
+    <t>Av. Javier Prado Este Nro. 4019</t>
+  </si>
+  <si>
+    <t>Ruc:</t>
+  </si>
+  <si>
+    <t>Fecha reporte:</t>
+  </si>
+  <si>
+    <t>usuario:</t>
+  </si>
+  <si>
+    <t>Nº GUIA DE REMISION REMITENTE</t>
+  </si>
+  <si>
+    <t>Nº GUIA DE REMISION TRANSPORTISTA</t>
+  </si>
+  <si>
+    <t>CÓDIGO</t>
+  </si>
+  <si>
+    <t>FECHA</t>
+  </si>
+  <si>
+    <t>TIPO MINERAL</t>
+  </si>
+  <si>
+    <t>UNIDAD MEDIDA</t>
+  </si>
+  <si>
+    <t>N° SACOS</t>
+  </si>
+  <si>
+    <t>CONSESION</t>
+  </si>
+  <si>
+    <t>MINERAL</t>
+  </si>
+  <si>
+    <t>Inter
+(US$ /Oz)</t>
+  </si>
+  <si>
+    <t>Ley 
+(Oz/TC)</t>
+  </si>
+  <si>
+    <t>Ley Cu
+%</t>
+  </si>
+  <si>
+    <t>Maquila
+(U$/ TC)</t>
+  </si>
+  <si>
+    <t>Recup. %</t>
+  </si>
+  <si>
+    <t>C.A.</t>
+  </si>
+  <si>
+    <t>Peso
+húmedo
+TM</t>
+  </si>
+  <si>
+    <t>Hum %</t>
+  </si>
+  <si>
+    <t>Peso Seco TM</t>
+  </si>
+  <si>
+    <t>Factor</t>
+  </si>
+  <si>
+    <t>Precio
+US $/TM</t>
+  </si>
+  <si>
+    <t>Precio
+Total
+US $</t>
+  </si>
+  <si>
+    <t>Proveedor:</t>
   </si>
 </sst>
 </file>
@@ -101,10 +125,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-&quot;S/&quot;\ * #,##0.00_-;\-&quot;S/&quot;\ * #,##0.00_-;_-&quot;S/&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;S/&quot;\ * #,##0.00_-;\-&quot;S/&quot;\ * #,##0.00_-;_-&quot;S/&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,6 +177,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -204,7 +241,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -218,7 +255,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -231,6 +268,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -277,9 +347,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -317,7 +387,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -423,7 +493,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -565,7 +635,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -573,15 +643,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0C1E24-7B74-4DAA-8B4C-375C7E9ECE99}">
-  <dimension ref="A1:BH5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BI10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="4" width="17.85546875" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.77734375" customWidth="1"/>
+    <col min="10" max="10" width="11.77734375" customWidth="1"/>
+    <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="21" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:61" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -642,31 +724,32 @@
       <c r="BF1" s="1"/>
       <c r="BG1" s="1"/>
       <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
     </row>
-    <row r="2" spans="1:60" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+    <row r="2" spans="1:61" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
       <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
@@ -706,29 +789,32 @@
       <c r="BF2" s="1"/>
       <c r="BG2" s="1"/>
       <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
     </row>
-    <row r="3" spans="1:60" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="1"/>
-      <c r="U3" s="1"/>
+    <row r="3" spans="1:61" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
@@ -768,95 +854,252 @@
       <c r="BF3" s="1"/>
       <c r="BG3" s="1"/>
       <c r="BH3" s="1"/>
+      <c r="BI3" s="1"/>
     </row>
-    <row r="4" spans="1:60" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
+    <row r="4" spans="1:61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="1"/>
+      <c r="Z4" s="1"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="1"/>
+      <c r="AC4" s="1"/>
+      <c r="AD4" s="1"/>
+      <c r="AE4" s="1"/>
+      <c r="AF4" s="1"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="1"/>
+      <c r="AI4" s="1"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="1"/>
+      <c r="AL4" s="1"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="1"/>
+      <c r="AO4" s="1"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
+      <c r="AS4" s="1"/>
+      <c r="AT4" s="1"/>
+      <c r="AU4" s="1"/>
+      <c r="AV4" s="1"/>
+      <c r="AW4" s="1"/>
+      <c r="AX4" s="1"/>
+      <c r="AY4" s="1"/>
+      <c r="AZ4" s="1"/>
+      <c r="BA4" s="1"/>
+      <c r="BB4" s="1"/>
+      <c r="BC4" s="1"/>
+      <c r="BD4" s="1"/>
+      <c r="BE4" s="1"/>
+      <c r="BF4" s="1"/>
+      <c r="BG4" s="1"/>
+      <c r="BH4" s="1"/>
+      <c r="BI4" s="1"/>
     </row>
-    <row r="5" spans="1:60" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:61" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+    </row>
+    <row r="6" spans="1:61" ht="18" x14ac:dyDescent="0.3">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+    </row>
+    <row r="7" spans="1:61" ht="18" x14ac:dyDescent="0.3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+    </row>
+    <row r="8" spans="1:61" ht="18" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+    </row>
+    <row r="9" spans="1:61" ht="18" x14ac:dyDescent="0.3">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+    </row>
+    <row r="10" spans="1:61" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="M10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="N5" s="3" t="s">
+      <c r="O10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="R5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="S5" s="3" t="s">
+      <c r="P10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="3" t="s">
-        <v>16</v>
+      <c r="Q10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A4:R4"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A5:I5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: guardar excel con celda activa en la primera fila
</commit_message>
<xml_diff>
--- a/liquidacion/analytica/Report/PreLiquidacion.xlsx
+++ b/liquidacion/analytica/Report/PreLiquidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\minersoft\acopio-project-configuration\liquidacion\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD5A92D-8B09-436A-8515-6929C4720338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24157AE6-86CB-428E-8367-21D4B4EF17B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
   </bookViews>
@@ -255,7 +255,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -297,6 +297,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -643,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0C1E24-7B74-4DAA-8B4C-375C7E9ECE99}">
-  <dimension ref="A1:BI10"/>
+  <dimension ref="A1:BI13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -727,17 +728,17 @@
       <c r="BI1" s="1"/>
     </row>
     <row r="2" spans="1:61" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
       <c r="J2" s="5"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -792,17 +793,17 @@
       <c r="BI2" s="1"/>
     </row>
     <row r="3" spans="1:61" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
       <c r="J3" s="7"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
@@ -920,17 +921,17 @@
       <c r="BI4" s="1"/>
     </row>
     <row r="5" spans="1:61" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
       <c r="J5" s="6"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
@@ -1095,6 +1096,14 @@
         <v>26</v>
       </c>
     </row>
+    <row r="13" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+      <c r="O13" s="15"/>
+      <c r="Q13" s="15"/>
+      <c r="U13" s="15"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:I2"/>

</xml_diff>

<commit_message>
feat: actualizar formato preliquidacion
</commit_message>
<xml_diff>
--- a/liquidacion/analytica/Report/PreLiquidacion.xlsx
+++ b/liquidacion/analytica/Report/PreLiquidacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\minersoft\acopio-project-configuration\liquidacion\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24157AE6-86CB-428E-8367-21D4B4EF17B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AC831D-D3C7-4403-A1EF-B0A57BDAA595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
+    <workbookView xWindow="4668" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>LIQUIDACION DE VENTA DE ACOPIO [el año  registro de la liquidación masiva]</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>Fecha reporte:</t>
-  </si>
-  <si>
-    <t>usuario:</t>
   </si>
   <si>
     <t>Nº GUIA DE REMISION REMITENTE</t>
@@ -118,6 +115,15 @@
   </si>
   <si>
     <t>Proveedor:</t>
+  </si>
+  <si>
+    <t>Creado por:</t>
+  </si>
+  <si>
+    <t>Fecha preliquidacion:</t>
+  </si>
+  <si>
+    <t>Exportado por:</t>
   </si>
 </sst>
 </file>
@@ -255,7 +261,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -298,6 +304,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -305,6 +314,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -658,7 +670,7 @@
     <col min="9" max="9" width="9.77734375" customWidth="1"/>
     <col min="10" max="10" width="11.77734375" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
     <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.5546875" bestFit="1" customWidth="1"/>
     <col min="15" max="21" width="11.6640625" customWidth="1"/>
@@ -728,17 +740,17 @@
       <c r="BI1" s="1"/>
     </row>
     <row r="2" spans="1:61" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
       <c r="J2" s="5"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -793,17 +805,17 @@
       <c r="BI2" s="1"/>
     </row>
     <row r="3" spans="1:61" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
       <c r="J3" s="7"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
@@ -921,17 +933,17 @@
       <c r="BI4" s="1"/>
     </row>
     <row r="5" spans="1:61" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
       <c r="J5" s="6"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
@@ -969,19 +981,21 @@
     <row r="7" spans="1:61" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K7" s="6"/>
+      <c r="L7" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -998,12 +1012,14 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="13" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
+      <c r="L8" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
@@ -1033,67 +1049,67 @@
     </row>
     <row r="10" spans="1:61" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="K10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="L10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="M10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="N10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="O10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="P10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="Q10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="Q10" s="3" t="s">
+      <c r="R10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="R10" s="3" t="s">
+      <c r="S10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="S10" s="3" t="s">
+      <c r="T10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="T10" s="3" t="s">
+      <c r="U10" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="U10" s="3" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:61" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat: ampliar ancho de columnas para reporte de preliquidacion
</commit_message>
<xml_diff>
--- a/liquidacion/analytica/Report/PreLiquidacion.xlsx
+++ b/liquidacion/analytica/Report/PreLiquidacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\minersoft\acopio-project-configuration\liquidacion\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AC831D-D3C7-4403-A1EF-B0A57BDAA595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD572573-875F-415F-8FAE-C253EF76DE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4668" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4948E9C5-4A82-4225-8782-1082295A0ACF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -261,7 +261,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -307,6 +307,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -316,8 +319,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -659,21 +668,27 @@
   <dimension ref="A1:BI13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" customWidth="1"/>
-    <col min="10" max="10" width="11.77734375" customWidth="1"/>
-    <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="21" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" customWidth="1"/>
+    <col min="6" max="6" width="28.44140625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5546875" customWidth="1"/>
+    <col min="9" max="9" width="24.77734375" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.109375" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="17.21875" customWidth="1"/>
+    <col min="15" max="15" width="15.5546875" customWidth="1"/>
+    <col min="16" max="16" width="15.33203125" customWidth="1"/>
+    <col min="17" max="17" width="11.109375" customWidth="1"/>
+    <col min="18" max="18" width="13.6640625" customWidth="1"/>
+    <col min="19" max="19" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:61" x14ac:dyDescent="0.3">
@@ -740,17 +755,17 @@
       <c r="BI1" s="1"/>
     </row>
     <row r="2" spans="1:61" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
       <c r="J2" s="5"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -805,17 +820,17 @@
       <c r="BI2" s="1"/>
     </row>
     <row r="3" spans="1:61" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
       <c r="J3" s="7"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
@@ -933,17 +948,17 @@
       <c r="BI4" s="1"/>
     </row>
     <row r="5" spans="1:61" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
       <c r="J5" s="6"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
@@ -983,19 +998,20 @@
       <c r="B7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="6"/>
+      <c r="C7" s="22"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="11" t="s">
         <v>28</v>
       </c>
+      <c r="H7" s="13"/>
       <c r="K7" s="6"/>
       <c r="L7" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="17"/>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -1014,12 +1030,13 @@
       <c r="G8" s="13" t="s">
         <v>27</v>
       </c>
+      <c r="H8" s="13"/>
       <c r="K8" s="6"/>
       <c r="L8" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="17"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
@@ -1112,6 +1129,7 @@
         <v>25</v>
       </c>
     </row>
+    <row r="11" spans="1:61" s="21" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:61" x14ac:dyDescent="0.3">
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>

</xml_diff>